<commit_message>
add: Extração da Leroy funcionando...
</commit_message>
<xml_diff>
--- a/data/default/prototipo_pluri.xlsx
+++ b/data/default/prototipo_pluri.xlsx
@@ -744,11 +744,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>

</xml_diff>